<commit_message>
docs(construcción/especificaciones): CU09 y CU20 terminados, CU12 avanzado
</commit_message>
<xml_diff>
--- a/Etapa Construcción - Iteración 1/Estimación 04 Caso Más Probable - Kairos - NexTech.xlsx
+++ b/Etapa Construcción - Iteración 1/Estimación 04 Caso Más Probable - Kairos - NexTech.xlsx
@@ -1068,7 +1068,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1257,7 +1257,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="9" fillId="3" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="4" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -1297,6 +1297,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="2" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="9" fillId="3" fontId="5" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4395,12 +4398,12 @@
       </c>
       <c r="D71" s="64">
         <f>IF($G$64&gt;=5,$G$71*(36/20),IF(AND($G$64&gt;2,$G$64&lt;=4),$G$71*(28/20), IF(AND($G$64&gt;=0,$G$64&lt;=2),$G$71,"error")))</f>
-        <v>2.8</v>
+        <v>4.382</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="1"/>
       <c r="G71" s="65">
-        <v>2.0</v>
+        <v>3.13</v>
       </c>
       <c r="H71" s="1"/>
       <c r="I71" s="1"/>
@@ -4466,7 +4469,7 @@
       </c>
       <c r="D73" s="63">
         <f t="shared" si="9"/>
-        <v>324.04736</v>
+        <v>507.1341184</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="1"/>
@@ -4505,7 +4508,7 @@
       </c>
       <c r="D74" s="69">
         <f>D73/(22*3)</f>
-        <v>4.909808485</v>
+        <v>7.683850279</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="1"/>
@@ -4674,7 +4677,7 @@
       </c>
       <c r="F79" s="68">
         <f t="shared" si="11"/>
-        <v>4.909808485</v>
+        <v>7.683850279</v>
       </c>
       <c r="G79" s="1"/>
       <c r="H79" s="1"/>
@@ -4716,7 +4719,7 @@
       </c>
       <c r="F80" s="63">
         <f t="shared" si="12"/>
-        <v>7.364712727</v>
+        <v>11.52577542</v>
       </c>
       <c r="G80" s="1"/>
       <c r="H80" s="1"/>
@@ -4756,7 +4759,7 @@
       </c>
       <c r="F81" s="68">
         <f t="shared" si="13"/>
-        <v>12.27452121</v>
+        <v>19.2096257</v>
       </c>
       <c r="G81" s="1"/>
       <c r="H81" s="1"/>
@@ -4915,7 +4918,7 @@
       </c>
       <c r="D86" s="77">
         <f>$F$81/$B$83</f>
-        <v>2.454904242</v>
+        <v>3.841925139</v>
       </c>
       <c r="E86" s="76"/>
       <c r="F86" s="76"/>
@@ -13858,7 +13861,7 @@
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="1"/>
-      <c r="G71" s="65">
+      <c r="G71" s="79">
         <v>2.0</v>
       </c>
       <c r="H71" s="1"/>
@@ -20714,16 +20717,16 @@
     <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B63:F63"/>
+    <mergeCell ref="B67:F67"/>
+    <mergeCell ref="B72:D72"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B50:F50"/>
     <mergeCell ref="B62:F62"/>
-    <mergeCell ref="B50:F50"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B72:D72"/>
-    <mergeCell ref="B67:F67"/>
-    <mergeCell ref="B63:F63"/>
-    <mergeCell ref="B49:F49"/>
   </mergeCells>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C8:C11">

</xml_diff>